<commit_message>
Planilhas de download: cabeçalho preto/branco (painel mantém as cores originais)
Ajusta build_downloads.py pra usar cabeçalho preto/branco nas planilhas
de "Baixar dados" — o pedido era só pro Excel, não pro painel (que foi
revertido pras cores institucionais no commit anterior).
</commit_message>
<xml_diff>
--- a/data/downloads/BNDES_2451.xlsx
+++ b/data/downloads/BNDES_2451.xlsx
@@ -30,6 +30,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="13"/>
     </font>
     <font>
@@ -39,6 +40,7 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00000000"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -55,9 +57,7 @@
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
-      </patternFill>
+      <patternFill patternType="solid"/>
     </fill>
   </fills>
   <borders count="2">

</xml_diff>